<commit_message>
Signatur-Logik aus E-Mail-Entwurf entfernt, .gitignore hinzugefügt
E-Mail-Entwürfe werden jetzt ohne automatische Signatur erstellt.
User wählt Signatur selbst in Outlook aus.
.gitignore für node_modules, .env und .DS_Store hinzugefügt.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bauvorhaben/_meta/Bauvorhaben.xlsx
+++ b/Bauvorhaben/_meta/Bauvorhaben.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>kuerzel</t>
   </si>
@@ -34,64 +34,25 @@
     <t>created_at</t>
   </si>
   <si>
-    <t>B-HB-RDR-04-25</t>
-  </si>
-  <si>
-    <t>KiTa Rudolf-Diesel-Ring</t>
-  </si>
-  <si>
-    <t>Max Mustermann</t>
-  </si>
-  <si>
-    <t>max@firma.at</t>
-  </si>
-  <si>
-    <t>cc@firma.at</t>
-  </si>
-  <si>
-    <t>Markt Holzkirchen</t>
-  </si>
-  <si>
-    <t>2026-01-25T18:53:00.332Z</t>
-  </si>
-  <si>
-    <t>HB-NORD-01</t>
-  </si>
-  <si>
-    <t>Umbau Nordhalle</t>
-  </si>
-  <si>
-    <t>Anna Huber</t>
-  </si>
-  <si>
-    <t>anna@firma.at</t>
-  </si>
-  <si>
-    <t>Stadt Muenchen</t>
-  </si>
-  <si>
-    <t>2026-01-25T18:58:03.157Z</t>
-  </si>
-  <si>
-    <t>SB-NORD-01</t>
-  </si>
-  <si>
-    <t>Baustelle sanierung</t>
-  </si>
-  <si>
-    <t>mehmet demir</t>
-  </si>
-  <si>
-    <t>demir@firma.at</t>
-  </si>
-  <si>
-    <t>kk@firma.at</t>
-  </si>
-  <si>
-    <t>Stadt Lindau</t>
-  </si>
-  <si>
-    <t>2026-01-25T19:30:26.594Z</t>
+    <t>SB-SÜD-02</t>
+  </si>
+  <si>
+    <t>Lindau Kindergarten</t>
+  </si>
+  <si>
+    <t>Sedat Demir</t>
+  </si>
+  <si>
+    <t>sedatfk38@gmail.com</t>
+  </si>
+  <si>
+    <t>sedat.demir@estably.com</t>
+  </si>
+  <si>
+    <t>Lindau</t>
+  </si>
+  <si>
+    <t>2026-03-10T17:03:54.965Z</t>
   </si>
 </sst>
 </file>
@@ -468,7 +429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -515,52 +476,6 @@
       </c>
       <c r="G2" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>